<commit_message>
chore(rename): frontend copy and metadata to Unde Labs
copy.name, the header wordmark, the share image, the Developers and
Accuracy pages, the API client's error strings and the BOM samples
(regenerated; ligatures off so the PDF text matches the old one).

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/samples/heatgun-bom.xlsx
+++ b/frontend/public/samples/heatgun-bom.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BOM" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="About" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="BOM" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="About" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1174,7 +1174,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Example test file for Origin Proof. Rows follow the facts of public CBP ruling N328954; company and part numbers are made up.</t>
+          <t>Example test file for Unde. Rows follow the facts of public CBP ruling N328954; company and part numbers are made up.</t>
         </is>
       </c>
     </row>

</xml_diff>